<commit_message>
adding thesis files and organizing
</commit_message>
<xml_diff>
--- a/data/Fall2018/db1-7_missing-data-runs/db5/15-genes_28-edges_db5_Sigmoid_estimation_missing-values.xlsx
+++ b/data/Fall2018/db1-7_missing-data-runs/db5/15-genes_28-edges_db5_Sigmoid_estimation_missing-values.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lmu0-my.sharepoint.com/personal/nchun2_lion_lmu_edu/Documents/Documents/GitHub/DahlquistLabTest/data/Fall2018/db1-7_missing-data-runs/db5/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_069524146986A3D8702BF85EDD1F0284761C6233" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9125BF4D-88D2-487F-9A48-D3B5CA8A2619}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23025" windowHeight="9375" tabRatio="877" firstSheet="2" activeTab="10"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="877" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="production_rates" sheetId="5" r:id="rId1"/>
@@ -20,8 +26,19 @@
     <sheet name="optimization_parameters" sheetId="9" r:id="rId11"/>
     <sheet name="threshold_b" sheetId="10" r:id="rId12"/>
   </sheets>
-  <calcPr calcId="145621" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
     </ext>
@@ -167,7 +184,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
@@ -218,7 +235,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -228,6 +245,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -606,7 +629,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -614,25 +637,22 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="277" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="277" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="277" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="277" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="277" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="277" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="277" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="277" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="277" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="277" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="348">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -982,7 +1002,7 @@
     <cellStyle name="Hyperlink" xfId="344" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="346" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 3" xfId="277"/>
+    <cellStyle name="Normal 3" xfId="277" xr:uid="{00000000-0005-0000-0000-00005B010000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
@@ -995,6 +1015,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1318,16 +1342,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.875" style="2"/>
+    <col min="1" max="1" width="10.8984375" style="2"/>
     <col min="2" max="2" width="14.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.875" style="2"/>
+    <col min="3" max="16384" width="10.8984375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
@@ -1335,7 +1359,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1343,7 +1367,7 @@
         <v>0.22359999999999999</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -1351,7 +1375,7 @@
         <v>0.43319999999999997</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1359,7 +1383,7 @@
         <v>0.2009</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -1367,7 +1391,7 @@
         <v>0.1925</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -1375,7 +1399,7 @@
         <v>0.32240000000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -1383,7 +1407,7 @@
         <v>0.27179999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -1391,7 +1415,7 @@
         <v>9.9000000000000005E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -1399,7 +1423,7 @@
         <v>0.40770000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -1407,7 +1431,7 @@
         <v>0.69310000000000005</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -1415,7 +1439,7 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -1423,7 +1447,7 @@
         <v>0.28289999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -1431,7 +1455,7 @@
         <v>0.32240000000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -1439,7 +1463,7 @@
         <v>0.17330000000000001</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -1447,7 +1471,7 @@
         <v>0.72960000000000003</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -1467,14 +1491,14 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:P16"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="10.875" style="2"/>
+    <col min="1" max="16384" width="10.8984375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>15</v>
       </c>
@@ -1524,7 +1548,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1574,7 +1598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -1624,7 +1648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1674,7 +1698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -1724,7 +1748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -1774,7 +1798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -1824,7 +1848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -1874,7 +1898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -1924,7 +1948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -1974,7 +1998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -2024,7 +2048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -2074,7 +2098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -2124,7 +2148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -2174,7 +2198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -2224,7 +2248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -2286,123 +2310,123 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:N16"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="10.875" style="2"/>
+    <col min="2" max="16384" width="10.8984375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="7">
         <v>2E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="7">
         <v>100000000</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="7">
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="7">
         <v>100000000</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="7">
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B9" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B12" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14" s="2">
         <v>15</v>
       </c>
       <c r="C14" s="2">
@@ -2412,17 +2436,17 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="2" t="s">
         <v>41</v>
       </c>
       <c r="E15" s="2" t="s">
@@ -2435,7 +2459,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>34</v>
       </c>
@@ -2491,14 +2515,14 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="10.875" style="2"/>
+    <col min="1" max="16384" width="10.8984375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
@@ -2506,7 +2530,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2514,7 +2538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -2522,7 +2546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -2530,7 +2554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -2538,7 +2562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -2546,7 +2570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -2554,7 +2578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -2562,7 +2586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -2570,7 +2594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -2578,7 +2602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -2586,7 +2610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -2594,7 +2618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -2602,7 +2626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -2610,7 +2634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -2618,7 +2642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -2638,16 +2662,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.875" style="2"/>
+    <col min="1" max="1" width="10.8984375" style="2"/>
     <col min="2" max="2" width="15.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.875" style="2"/>
+    <col min="3" max="16384" width="10.8984375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
@@ -2655,7 +2679,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2663,7 +2687,7 @@
         <v>0.1118</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -2671,7 +2695,7 @@
         <v>0.21659999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -2679,7 +2703,7 @@
         <v>0.10050000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -2687,7 +2711,7 @@
         <v>9.6299999999999997E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -2695,7 +2719,7 @@
         <v>0.16120000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -2703,7 +2727,7 @@
         <v>0.13589999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -2711,7 +2735,7 @@
         <v>4.9500000000000002E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -2719,7 +2743,7 @@
         <v>0.2039</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -2727,7 +2751,7 @@
         <v>0.34660000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -2735,7 +2759,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -2743,7 +2767,7 @@
         <v>0.14149999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -2751,7 +2775,7 @@
         <v>0.16120000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -2759,7 +2783,7 @@
         <v>8.6599999999999996E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -2767,7 +2791,7 @@
         <v>0.36480000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -2787,14 +2811,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:N17"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="10.875" style="2"/>
+    <col min="1" max="16384" width="10.8984375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
@@ -2838,7 +2862,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2880,7 +2904,7 @@
         <v>-1.2497</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -2924,7 +2948,7 @@
         <v>-0.92479999999999996</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -2968,7 +2992,7 @@
         <v>1.4784999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -3012,7 +3036,7 @@
         <v>-0.35849999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -3056,7 +3080,7 @@
         <v>0.1953</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -3100,7 +3124,7 @@
         <v>-1.8463000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -3144,7 +3168,7 @@
         <v>2.2172000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -3188,7 +3212,7 @@
         <v>-0.12709999999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -3232,7 +3256,7 @@
         <v>-1.0367</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -3276,7 +3300,7 @@
         <v>-0.27479999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -3320,7 +3344,7 @@
         <v>0.28120000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -3364,7 +3388,7 @@
         <v>9.7000000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -3408,7 +3432,7 @@
         <v>-0.72499999999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -3452,7 +3476,7 @@
         <v>-0.51170000000000004</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -3494,7 +3518,7 @@
       </c>
       <c r="N16" s="4"/>
     </row>
-    <row r="17" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G17" s="3"/>
     </row>
   </sheetData>
@@ -3509,14 +3533,14 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:N17"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="10.875" style="2"/>
+    <col min="1" max="16384" width="10.8984375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
@@ -3558,46 +3582,46 @@
       </c>
       <c r="N1" s="1"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="11">
+      <c r="B2" s="8">
         <v>-0.17180000000000001</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="9">
         <v>-0.2792</v>
       </c>
-      <c r="D2" s="11">
+      <c r="D2" s="8">
         <v>-0.17519999999999999</v>
       </c>
-      <c r="E2" s="11">
+      <c r="E2" s="8">
         <v>-0.68840000000000001</v>
       </c>
-      <c r="F2" s="12">
+      <c r="F2" s="9">
         <v>-0.24360000000000001</v>
       </c>
-      <c r="G2" s="12">
+      <c r="G2" s="9">
         <v>0.15809999999999999</v>
       </c>
-      <c r="H2" s="11">
+      <c r="H2" s="8">
         <v>-0.42530000000000001</v>
       </c>
-      <c r="I2" s="13"/>
-      <c r="J2" s="11">
+      <c r="I2" s="10"/>
+      <c r="J2" s="8">
         <v>0.56820000000000004</v>
       </c>
-      <c r="K2" s="11">
+      <c r="K2" s="8">
         <v>0.1646</v>
       </c>
-      <c r="L2" s="11">
+      <c r="L2" s="8">
         <v>-0.32019999999999998</v>
       </c>
-      <c r="M2" s="11">
+      <c r="M2" s="8">
         <v>-0.38879999999999998</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -3638,167 +3662,167 @@
         <v>-1.3284</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="8">
         <v>-0.66849999999999998</v>
       </c>
-      <c r="C4" s="14"/>
-      <c r="D4" s="11">
+      <c r="C4" s="11"/>
+      <c r="D4" s="8">
         <v>-0.43219999999999997</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="8">
         <v>-0.1191</v>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="9">
         <v>-0.38300000000000001</v>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="9">
         <v>0.26929999999999998</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="8">
         <v>-7.5700000000000003E-2</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I4" s="8">
         <v>0.59750000000000003</v>
       </c>
-      <c r="J4" s="13"/>
-      <c r="K4" s="11">
+      <c r="J4" s="10"/>
+      <c r="K4" s="8">
         <v>-0.3216</v>
       </c>
-      <c r="L4" s="11">
+      <c r="L4" s="8">
         <v>8.0500000000000002E-2</v>
       </c>
-      <c r="M4" s="11">
+      <c r="M4" s="8">
         <v>0.4778</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="8">
         <v>-0.3155</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="9">
         <v>1.4649000000000001</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="8">
         <v>-0.80289999999999995</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="8">
         <v>0.5141</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="9">
         <v>-0.76539999999999997</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="9">
         <v>-1.1456</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="8">
         <v>0.50960000000000005</v>
       </c>
-      <c r="I5" s="11">
+      <c r="I5" s="8">
         <v>-0.29570000000000002</v>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="8">
         <v>-0.22570000000000001</v>
       </c>
-      <c r="K5" s="11">
+      <c r="K5" s="8">
         <v>-0.94040000000000001</v>
       </c>
-      <c r="L5" s="11">
+      <c r="L5" s="8">
         <v>-1.3326</v>
       </c>
-      <c r="M5" s="11">
+      <c r="M5" s="8">
         <v>0.16889999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="8">
         <v>0.96209999999999996</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="9">
         <v>-0.3518</v>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="8">
         <v>0.31009999999999999</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="8">
         <v>-0.15890000000000001</v>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="9">
         <v>0.58689999999999998</v>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="9">
         <v>3.4099999999999998E-2</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="8">
         <v>0.48599999999999999</v>
       </c>
-      <c r="I6" s="11">
+      <c r="I6" s="8">
         <v>0.43419999999999997</v>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="8">
         <v>1.0717000000000001</v>
       </c>
-      <c r="K6" s="15">
+      <c r="K6" s="12">
         <v>5.5899999999999998E-2</v>
       </c>
-      <c r="L6" s="11">
+      <c r="L6" s="8">
         <v>1.1548</v>
       </c>
-      <c r="M6" s="11">
+      <c r="M6" s="8">
         <v>0.54459999999999997</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="8">
         <v>6.3299999999999995E-2</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="9">
         <v>0.17119999999999999</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="8">
         <v>-1.9531000000000001</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="8">
         <v>-0.21510000000000001</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="9">
         <v>-1.4630000000000001</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="9">
         <v>0.30249999999999999</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="8">
         <v>-2.2646000000000002</v>
       </c>
-      <c r="I7" s="11">
+      <c r="I7" s="8">
         <v>1.4417</v>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="8">
         <v>-1.2318</v>
       </c>
-      <c r="K7" s="11">
+      <c r="K7" s="8">
         <v>-0.14030000000000001</v>
       </c>
-      <c r="L7" s="11">
+      <c r="L7" s="8">
         <v>-1.9814000000000001</v>
       </c>
-      <c r="M7" s="11">
+      <c r="M7" s="8">
         <v>-1.2117</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -3839,46 +3863,46 @@
         <v>1.4664999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="12">
+      <c r="B9" s="13"/>
+      <c r="C9" s="9">
         <v>-0.54890000000000005</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="8">
         <v>0.24909999999999999</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="8">
         <v>0.90359999999999996</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="9">
         <v>-0.5302</v>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="9">
         <v>1.6E-2</v>
       </c>
-      <c r="H9" s="11">
+      <c r="H9" s="8">
         <v>-9.9699999999999997E-2</v>
       </c>
-      <c r="I9" s="11">
+      <c r="I9" s="8">
         <v>1.0787</v>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="8">
         <v>-0.1371</v>
       </c>
-      <c r="K9" s="11">
+      <c r="K9" s="8">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="L9" s="11">
+      <c r="L9" s="8">
         <v>0.40110000000000001</v>
       </c>
-      <c r="M9" s="11">
+      <c r="M9" s="8">
         <v>6.0299999999999999E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -3919,7 +3943,7 @@
         <v>0.31269999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -3960,14 +3984,14 @@
         <v>1.1318999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B12" s="2">
         <v>-0.4763</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="14">
         <v>-0.45290000000000002</v>
       </c>
       <c r="D12" s="2">
@@ -4001,7 +4025,7 @@
         <v>0.23119999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -4042,7 +4066,7 @@
         <v>0.20899999999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -4083,7 +4107,7 @@
         <v>0.55789999999999995</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -4124,48 +4148,48 @@
         <v>0.29849999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="8">
         <v>0.83440000000000003</v>
       </c>
-      <c r="C16" s="12">
+      <c r="C16" s="9">
         <v>0.83979999999999999</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="8">
         <v>0.91839999999999999</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="8">
         <v>0.47470000000000001</v>
       </c>
-      <c r="F16" s="12">
+      <c r="F16" s="9">
         <v>2.3845000000000001</v>
       </c>
-      <c r="G16" s="12">
+      <c r="G16" s="9">
         <v>0.1525</v>
       </c>
-      <c r="H16" s="11">
+      <c r="H16" s="8">
         <v>0.65110000000000001</v>
       </c>
-      <c r="I16" s="11">
+      <c r="I16" s="8">
         <v>-0.82630000000000003</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J16" s="8">
         <v>0.31130000000000002</v>
       </c>
-      <c r="K16" s="11">
+      <c r="K16" s="8">
         <v>-9.06E-2</v>
       </c>
-      <c r="L16" s="11">
+      <c r="L16" s="8">
         <v>0.96989999999999998</v>
       </c>
-      <c r="M16" s="11">
+      <c r="M16" s="8">
         <v>-4.41E-2</v>
       </c>
     </row>
-    <row r="17" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G17" s="3"/>
     </row>
   </sheetData>
@@ -4180,14 +4204,14 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:N16"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="10.875" style="2"/>
+    <col min="1" max="16384" width="10.8984375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
@@ -4229,7 +4253,7 @@
       </c>
       <c r="N1" s="1"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -4270,7 +4294,7 @@
         <v>-0.1933</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -4311,7 +4335,7 @@
         <v>-1.3101</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -4352,7 +4376,7 @@
         <v>2.5788000000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -4391,7 +4415,7 @@
         <v>0.76729999999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -4432,7 +4456,7 @@
         <v>-0.161</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -4473,7 +4497,7 @@
         <v>0.22559999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -4514,7 +4538,7 @@
         <v>1.7134</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -4555,7 +4579,7 @@
         <v>-0.28699999999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -4596,7 +4620,7 @@
         <v>1.2221</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -4635,7 +4659,7 @@
         <v>0.2671</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -4676,7 +4700,7 @@
         <v>-0.27239999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -4715,7 +4739,7 @@
         <v>0.2162</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -4756,7 +4780,7 @@
         <v>1.0390999999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -4795,7 +4819,7 @@
         <v>1.2979000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -4842,14 +4866,14 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:N17"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="10.875" style="2"/>
+    <col min="1" max="16384" width="10.8984375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
@@ -4891,7 +4915,7 @@
       </c>
       <c r="N1" s="1"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -4932,7 +4956,7 @@
         <v>0.19850000000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -4973,7 +4997,7 @@
         <v>-1.5982000000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -5014,7 +5038,7 @@
         <v>1.9187000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -5055,7 +5079,7 @@
         <v>0.95779999999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -5096,7 +5120,7 @@
         <v>1.0246</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -5137,7 +5161,7 @@
         <v>-0.52849999999999997</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -5178,7 +5202,7 @@
         <v>-0.2676</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -5219,7 +5243,7 @@
         <v>0.34039999999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -5260,7 +5284,7 @@
         <v>0.45229999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -5295,7 +5319,7 @@
         <v>0.16170000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -5334,7 +5358,7 @@
         <v>0.20960000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -5373,7 +5397,7 @@
         <v>0.72799999999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -5414,7 +5438,7 @@
         <v>0.97740000000000005</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -5455,7 +5479,7 @@
         <v>-1.0412999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -5494,7 +5518,7 @@
         <v>-0.5958</v>
       </c>
     </row>
-    <row r="17" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G17" s="3"/>
     </row>
   </sheetData>
@@ -5509,14 +5533,14 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:N16"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="10.875" style="2"/>
+    <col min="1" max="16384" width="10.8984375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
@@ -5558,7 +5582,7 @@
       </c>
       <c r="N1" s="1"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -5599,7 +5623,7 @@
         <v>-0.23880000000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -5640,7 +5664,7 @@
         <v>-0.87539999999999996</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -5681,7 +5705,7 @@
         <v>1.0147999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -5722,7 +5746,7 @@
         <v>-0.80569999999999997</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -5763,7 +5787,7 @@
         <v>0.89139999999999997</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -5804,7 +5828,7 @@
         <v>-0.88439999999999996</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -5845,7 +5869,7 @@
         <v>0.46439999999999998</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -5886,7 +5910,7 @@
         <v>0.57889999999999997</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -5927,7 +5951,7 @@
         <v>-0.58509999999999995</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -5958,7 +5982,7 @@
       <c r="L11" s="5"/>
       <c r="M11" s="5"/>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -5999,7 +6023,7 @@
         <v>0.52290000000000003</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -6040,7 +6064,7 @@
         <v>-0.54159999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -6081,7 +6105,7 @@
         <v>0.14030000000000001</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -6122,7 +6146,7 @@
         <v>-2.0924</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -6175,14 +6199,14 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:N16"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="10.875" style="2"/>
+    <col min="1" max="16384" width="10.8984375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
@@ -6224,7 +6248,7 @@
       </c>
       <c r="N1" s="1"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -6265,7 +6289,7 @@
         <v>-0.53690000000000004</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -6306,7 +6330,7 @@
         <v>-1.2416</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -6345,7 +6369,7 @@
         <v>2.6749999999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -6386,7 +6410,7 @@
         <v>0.6109</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -6427,7 +6451,7 @@
         <v>1.0084</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -6468,7 +6492,7 @@
         <v>-1.1214</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -6509,7 +6533,7 @@
         <v>2.0417000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -6550,7 +6574,7 @@
         <v>0.84799999999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -6581,7 +6605,7 @@
       <c r="J10" s="2">
         <v>-0.68630000000000002</v>
       </c>
-      <c r="K10" s="17">
+      <c r="K10" s="7">
         <v>1E-4</v>
       </c>
       <c r="L10" s="2">
@@ -6591,7 +6615,7 @@
         <v>0.55059999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -6632,7 +6656,7 @@
         <v>0.19139999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -6673,7 +6697,7 @@
         <v>0.2419</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -6714,7 +6738,7 @@
         <v>-0.28360000000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -6755,7 +6779,7 @@
         <v>0.69569999999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -6796,7 +6820,7 @@
         <v>-1.0581</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -6845,14 +6869,14 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:P16"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="10.875" style="2"/>
+    <col min="1" max="16384" width="10.8984375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>15</v>
       </c>
@@ -6902,7 +6926,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -6952,7 +6976,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -7002,7 +7026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -7052,7 +7076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -7102,7 +7126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -7152,7 +7176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -7202,7 +7226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -7252,7 +7276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -7302,7 +7326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -7352,7 +7376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -7402,7 +7426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -7452,7 +7476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -7502,7 +7526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -7552,7 +7576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -7602,7 +7626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>

</xml_diff>